<commit_message>
Fix recurring display layout and future filtering
</commit_message>
<xml_diff>
--- a/טרנזקציות חיובים קבועים לטעינה באפריל 2026.xlsx
+++ b/טרנזקציות חיובים קבועים לטעינה באפריל 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Shay\Trackly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{55A91003-4DF7-42C7-A8E8-5F0E0546AD6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15740FCB-0B37-4A1B-A9B8-C7EA63B795F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="720" windowWidth="14610" windowHeight="15480" xr2:uid="{B369152B-0B35-47A7-9405-4A875B8D3037}"/>
+    <workbookView xWindow="1560" yWindow="0" windowWidth="14610" windowHeight="15480" xr2:uid="{B369152B-0B35-47A7-9405-4A875B8D3037}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="43">
   <si>
     <t>id</t>
   </si>
@@ -62,36 +62,6 @@
     <t>description</t>
   </si>
   <si>
-    <t>date</t>
-  </si>
-  <si>
-    <t>installments</t>
-  </si>
-  <si>
-    <t>recurrence</t>
-  </si>
-  <si>
-    <t>installment_group_id</t>
-  </si>
-  <si>
-    <t>installment_index</t>
-  </si>
-  <si>
-    <t>installment_total</t>
-  </si>
-  <si>
-    <t>recurrence_group_id</t>
-  </si>
-  <si>
-    <t>recurrence_index</t>
-  </si>
-  <si>
-    <t>recurrence_total</t>
-  </si>
-  <si>
-    <t>is_deleted</t>
-  </si>
-  <si>
     <t>created_date</t>
   </si>
   <si>
@@ -144,16 +114,77 @@
   </si>
   <si>
     <t>Google one</t>
+  </si>
+  <si>
+    <t>random-id-001</t>
+  </si>
+  <si>
+    <t>random-id-002</t>
+  </si>
+  <si>
+    <t>random-id-003</t>
+  </si>
+  <si>
+    <t>random-id-004</t>
+  </si>
+  <si>
+    <t>random-id-005</t>
+  </si>
+  <si>
+    <t>random-id-006</t>
+  </si>
+  <si>
+    <t>random-id-007</t>
+  </si>
+  <si>
+    <t>random-id-008</t>
+  </si>
+  <si>
+    <t>random-id-009</t>
+  </si>
+  <si>
+    <t>random-id-010</t>
+  </si>
+  <si>
+    <t>random-id-011</t>
+  </si>
+  <si>
+    <t>random-id-012</t>
+  </si>
+  <si>
+    <t>random-id-013</t>
+  </si>
+  <si>
+    <t>random-id-014</t>
+  </si>
+  <si>
+    <t>day_of_month</t>
+  </si>
+  <si>
+    <t>is_active</t>
+  </si>
+  <si>
+    <t>start_date</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="177"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="177"/>
@@ -180,9 +211,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,10 +529,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{494A1486-544C-4F7D-8190-44505117CDE6}">
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="9.875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -514,497 +552,562 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
       <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C2">
         <v>24</v>
       </c>
-      <c r="D2">
-        <v>5</v>
+      <c r="D2" t="s">
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" s="1">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="2">
         <v>46117</v>
       </c>
-      <c r="R2" t="b">
-        <v>0</v>
-      </c>
-      <c r="S2" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K2">
+        <v>5</v>
+      </c>
+      <c r="L2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C3">
         <v>5</v>
       </c>
-      <c r="D3">
-        <v>5</v>
+      <c r="D3" t="s">
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3">
-        <v>13</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="1">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="2">
         <v>46117</v>
       </c>
-      <c r="R3" t="b">
-        <v>0</v>
-      </c>
-      <c r="S3" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>10</v>
       </c>
-      <c r="D4">
-        <v>5</v>
+      <c r="D4" t="s">
+        <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4">
-        <v>13</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" s="1">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="2">
         <v>46118</v>
       </c>
-      <c r="R4" t="b">
-        <v>0</v>
-      </c>
-      <c r="S4" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H4">
+        <v>6</v>
+      </c>
+      <c r="I4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K4">
+        <v>5</v>
+      </c>
+      <c r="L4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>52</v>
       </c>
-      <c r="D5">
-        <v>5</v>
+      <c r="D5" t="s">
+        <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5">
-        <v>13</v>
-      </c>
-      <c r="G5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I5" s="1">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="2">
         <v>46119</v>
       </c>
-      <c r="R5" t="b">
-        <v>0</v>
-      </c>
-      <c r="S5" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K5">
+        <v>5</v>
+      </c>
+      <c r="L5">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C6">
         <v>17</v>
       </c>
-      <c r="D6">
-        <v>5</v>
+      <c r="D6" t="s">
+        <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="1">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="2">
         <v>46122</v>
       </c>
-      <c r="R6" t="b">
-        <v>0</v>
-      </c>
-      <c r="S6" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C7">
         <v>12</v>
       </c>
-      <c r="D7">
-        <v>5</v>
+      <c r="D7" t="s">
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I7" s="1">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="2">
         <v>46123</v>
       </c>
-      <c r="R7" t="b">
-        <v>0</v>
-      </c>
-      <c r="S7" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H7">
+        <v>11</v>
+      </c>
+      <c r="I7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K7">
+        <v>5</v>
+      </c>
+      <c r="L7">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
-      <c r="D8">
-        <v>5</v>
+      <c r="D8" t="s">
+        <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8">
-        <v>13</v>
-      </c>
-      <c r="G8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I8" s="1">
+        <v>11</v>
+      </c>
+      <c r="F8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="2">
         <v>46123</v>
       </c>
-      <c r="R8" t="b">
-        <v>0</v>
-      </c>
-      <c r="S8" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H8">
+        <v>11</v>
+      </c>
+      <c r="I8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K8">
+        <v>5</v>
+      </c>
+      <c r="L8">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C9">
         <v>65</v>
       </c>
-      <c r="D9">
-        <v>5</v>
+      <c r="D9" t="s">
+        <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9">
-        <v>13</v>
-      </c>
-      <c r="G9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H9" t="s">
-        <v>29</v>
-      </c>
-      <c r="I9" s="1">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="2">
         <v>46126</v>
       </c>
-      <c r="R9" t="b">
-        <v>0</v>
-      </c>
-      <c r="S9" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H9">
+        <v>14</v>
+      </c>
+      <c r="I9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K9">
+        <v>5</v>
+      </c>
+      <c r="L9">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C10">
         <v>70</v>
       </c>
-      <c r="D10">
-        <v>5</v>
+      <c r="D10" t="s">
+        <v>10</v>
       </c>
       <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" t="s">
         <v>20</v>
       </c>
-      <c r="F10">
-        <v>13</v>
-      </c>
-      <c r="G10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H10" t="s">
-        <v>30</v>
-      </c>
-      <c r="I10" s="1">
+      <c r="G10" s="2">
         <v>46126</v>
       </c>
-      <c r="R10" t="b">
-        <v>0</v>
-      </c>
-      <c r="S10" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H10">
+        <v>14</v>
+      </c>
+      <c r="I10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K10">
+        <v>5</v>
+      </c>
+      <c r="L10">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C11">
         <v>65</v>
       </c>
-      <c r="D11">
-        <v>5</v>
+      <c r="D11" t="s">
+        <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F11">
-        <v>13</v>
-      </c>
-      <c r="G11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" t="s">
         <v>21</v>
       </c>
-      <c r="H11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I11" s="1">
+      <c r="G11" s="2">
         <v>46128</v>
       </c>
-      <c r="R11" t="b">
-        <v>0</v>
-      </c>
-      <c r="S11" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H11">
+        <v>16</v>
+      </c>
+      <c r="I11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K11">
+        <v>5</v>
+      </c>
+      <c r="L11">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C12">
         <v>298</v>
       </c>
-      <c r="D12">
-        <v>5</v>
+      <c r="D12" t="s">
+        <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>20</v>
-      </c>
-      <c r="F12">
+        <v>22</v>
+      </c>
+      <c r="G12" s="2">
+        <v>46134</v>
+      </c>
+      <c r="H12">
+        <v>22</v>
+      </c>
+      <c r="I12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K12">
+        <v>5</v>
+      </c>
+      <c r="L12">
         <v>14</v>
       </c>
-      <c r="G12" t="s">
-        <v>32</v>
-      </c>
-      <c r="I12" s="1">
-        <v>46134</v>
-      </c>
-      <c r="R12" t="b">
-        <v>0</v>
-      </c>
-      <c r="S12" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C13">
         <v>40</v>
       </c>
-      <c r="D13">
-        <v>5</v>
+      <c r="D13" t="s">
+        <v>10</v>
       </c>
       <c r="E13" t="s">
-        <v>20</v>
-      </c>
-      <c r="F13">
-        <v>13</v>
-      </c>
-      <c r="G13" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" t="s">
-        <v>33</v>
-      </c>
-      <c r="I13" s="1">
+        <v>11</v>
+      </c>
+      <c r="F13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G13" s="2">
         <v>46136</v>
       </c>
-      <c r="R13" t="b">
-        <v>0</v>
-      </c>
-      <c r="S13" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H13">
+        <v>24</v>
+      </c>
+      <c r="I13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K13">
+        <v>5</v>
+      </c>
+      <c r="L13">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C14">
         <v>10</v>
       </c>
-      <c r="D14">
-        <v>5</v>
+      <c r="D14" t="s">
+        <v>10</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14">
-        <v>13</v>
-      </c>
-      <c r="G14" t="s">
-        <v>21</v>
-      </c>
-      <c r="H14" t="s">
-        <v>34</v>
-      </c>
-      <c r="I14" s="1">
+        <v>11</v>
+      </c>
+      <c r="F14" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" s="2">
         <v>46139</v>
       </c>
-      <c r="R14" t="b">
-        <v>0</v>
-      </c>
-      <c r="S14" s="1">
-        <v>46137</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H14">
+        <v>27</v>
+      </c>
+      <c r="I14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J14" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K14">
+        <v>5</v>
+      </c>
+      <c r="L14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C15">
         <v>7</v>
       </c>
-      <c r="D15">
-        <v>5</v>
+      <c r="D15" t="s">
+        <v>10</v>
       </c>
       <c r="E15" t="s">
-        <v>20</v>
-      </c>
-      <c r="F15">
-        <v>13</v>
-      </c>
-      <c r="G15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H15" t="s">
-        <v>35</v>
-      </c>
-      <c r="I15" s="1">
+        <v>11</v>
+      </c>
+      <c r="F15" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="2">
         <v>46141</v>
       </c>
-      <c r="R15" t="b">
-        <v>0</v>
-      </c>
-      <c r="S15" s="1">
-        <v>46137</v>
+      <c r="H15">
+        <v>29</v>
+      </c>
+      <c r="I15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" s="2">
+        <v>46138</v>
+      </c>
+      <c r="K15">
+        <v>5</v>
+      </c>
+      <c r="L15">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>